<commit_message>
Update children database and Cloudflare seed
</commit_message>
<xml_diff>
--- a/База детей.xlsx
+++ b/База детей.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/k_r_kisanov/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/k_r_kisanov/Desktop/ProjectCodex/tg bot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A148C2-2D86-B046-A7FD-45F59E00710E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93C5C2C-53A0-4341-9B11-6897301A4E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1958" uniqueCount="1105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2198" uniqueCount="1214">
   <si>
     <t>ФИО ребёнка</t>
   </si>
@@ -3335,6 +3335,333 @@
   </si>
   <si>
     <t>Темирбекова  Кира Канатовна</t>
+  </si>
+  <si>
+    <t>Усеин Айару Талғатқызы</t>
+  </si>
+  <si>
+    <t>Шабхатова Айсарабану Шерикбайқызы</t>
+  </si>
+  <si>
+    <t>Умирханова Жания Жомартовна</t>
+  </si>
+  <si>
+    <t>Алиева Мунавар Камрановна</t>
+  </si>
+  <si>
+    <t>Азамат Медина</t>
+  </si>
+  <si>
+    <t>Алиева Амина Камрановна</t>
+  </si>
+  <si>
+    <t>Усеин Әдемі Талғатқызы</t>
+  </si>
+  <si>
+    <t>Асан Медина Жалғасқызы</t>
+  </si>
+  <si>
+    <t>Матвиенко Ариана Александровна</t>
+  </si>
+  <si>
+    <t>Асан Бибіфатима Жалғасқызы</t>
+  </si>
+  <si>
+    <t>Шабхатова Салиха Шерикбаевна</t>
+  </si>
+  <si>
+    <t>Дадаханова  Зухра Бобировна</t>
+  </si>
+  <si>
+    <t>Алиева Айгул Нурдавлатовна</t>
+  </si>
+  <si>
+    <t>Алиева Амина Нурдавлатовна</t>
+  </si>
+  <si>
+    <t>Усеин Каусар Талғатқызы</t>
+  </si>
+  <si>
+    <t>Анарбаев Рахимжон Юлдашович</t>
+  </si>
+  <si>
+    <t>Азизов Айдын Махмудович</t>
+  </si>
+  <si>
+    <t>Өтеген Айару Нұрмаханқызы</t>
+  </si>
+  <si>
+    <t>Исмаил Эмруллах Нурмамәдұлы</t>
+  </si>
+  <si>
+    <t>Исмаил Айлин Нурмамәдқызы</t>
+  </si>
+  <si>
+    <t>Кульбекова Венера Асхатовна</t>
+  </si>
+  <si>
+    <t>Бимурза Жанерке Жанәділқызы</t>
+  </si>
+  <si>
+    <t>Беймырза Ақниет Жангелдіқызы</t>
+  </si>
+  <si>
+    <t>Қайрат Нұрислам Нұрсұлтанұлы</t>
+  </si>
+  <si>
+    <t>Өтеген Рауан Нұрмаханқызы</t>
+  </si>
+  <si>
+    <t>Өмірхан Бекнұр Жомартұлы</t>
+  </si>
+  <si>
+    <t>Ескерәлі Үміт Темірәліқызы</t>
+  </si>
+  <si>
+    <t>Орынбасар Алихан Мадиярұлы</t>
+  </si>
+  <si>
+    <t>Ибадулла Айнұр Баймұратқызы</t>
+  </si>
+  <si>
+    <t>Даврушов Нурислам Асланович</t>
+  </si>
+  <si>
+    <t>Азамат Асель</t>
+  </si>
+  <si>
+    <t>Утеген  Саян  Нұрмаханұлы</t>
+  </si>
+  <si>
+    <t>Матвиенко Александр Васильевич</t>
+  </si>
+  <si>
+    <t>Матвиенко София Александровна</t>
+  </si>
+  <si>
+    <t>Жанділла Омар Баймұратұлы</t>
+  </si>
+  <si>
+    <t>Даврушов Азиз Асланұлы</t>
+  </si>
+  <si>
+    <t>Тұрысжан Айсұлтан Нұрланұлы</t>
+  </si>
+  <si>
+    <t>Тұрысжан Айгерім Нұрланқызы</t>
+  </si>
+  <si>
+    <t>Беимурза Жанасыл Жанәділұлы</t>
+  </si>
+  <si>
+    <t>Анарбаев Рамазан Юлдашович</t>
+  </si>
+  <si>
+    <t>АЙХАН ТАНИБЕРГЕНОВА АЙТМУХАМЕДОВНА</t>
+  </si>
+  <si>
+    <t>УМСИНАЙ МАТКАСИМОВА КАМАЛОВНА</t>
+  </si>
+  <si>
+    <t>АЙГУЛЬ ТЕМИРБАЕВА ХАНАЛБЕКОВНА</t>
+  </si>
+  <si>
+    <t>БАЛАХАНЫМ АЛИЕВА БАДЫРҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>ГУЛЖАН МУХАНБЕТОВА НАБИЕВНА</t>
+  </si>
+  <si>
+    <t>АЯНА ДҮКЕНБАЙ БИНАЗАРҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>ГАЛИНА МЕЛЬНИКОВА ДИМИТРИЕВНА</t>
+  </si>
+  <si>
+    <t>БОБИР АБДУЛЛАЕВ ДАДАХАНОВИЧ</t>
+  </si>
+  <si>
+    <t>РАЙЛА АЛИЕВА АГАЛИЕВНА</t>
+  </si>
+  <si>
+    <t>ФЕРУЗА РАМЕТОВА ХАКРАМАНҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>РАИЛЯ АЗИЗОВА РАШИДОВНА</t>
+  </si>
+  <si>
+    <t>АЙГЕРИМ СЫЗДИКОВА КАСИМБЕТОВНА</t>
+  </si>
+  <si>
+    <t>ЗУЛӘЛ ИСМАИЛОВА АЛИСУЛТАНҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>МОЛДИР ТАМПИШЕВА СЕРИКОВНА</t>
+  </si>
+  <si>
+    <t>МАИРА КАДЫРБАЕВА КАДИРБАЕВНА</t>
+  </si>
+  <si>
+    <t>ЖАЙНА КАДЫРБАЕВА ӘБІЛТАЙҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>НАЗГУЛ ҒАППАРОВА МҰХТАРҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>ИНДИРА АЛИШОВА ШУКИРДИНОВНА</t>
+  </si>
+  <si>
+    <t>УЛДАНА АЙМБЕТОВА ЕРАЛИЕВНА</t>
+  </si>
+  <si>
+    <t>ҚҰРАЛАЙ НҰРЖАН НӘЛІБЕКҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>НИГАРА КУЛИЕВА КАРИМОВНА</t>
+  </si>
+  <si>
+    <t>ДАМИРА МАТВИЕНКО ТОЛЕУОВНА</t>
+  </si>
+  <si>
+    <t>АЙСҰЛУ ТӨЛЕНДІ ТЕКЕБАЙҚЫЗЫ</t>
+  </si>
+  <si>
+    <t>87022021182</t>
+  </si>
+  <si>
+    <t>930103499059</t>
+  </si>
+  <si>
+    <t>87013722807</t>
+  </si>
+  <si>
+    <t>860304402300</t>
+  </si>
+  <si>
+    <t>87009571567</t>
+  </si>
+  <si>
+    <t>730423401432</t>
+  </si>
+  <si>
+    <t>87752751492</t>
+  </si>
+  <si>
+    <t>951010401247</t>
+  </si>
+  <si>
+    <t>87784348656</t>
+  </si>
+  <si>
+    <t>890127402473</t>
+  </si>
+  <si>
+    <t>87025274499</t>
+  </si>
+  <si>
+    <t>990106400196</t>
+  </si>
+  <si>
+    <t>87761992851</t>
+  </si>
+  <si>
+    <t>980728400453</t>
+  </si>
+  <si>
+    <t>87023354751</t>
+  </si>
+  <si>
+    <t>890524302019</t>
+  </si>
+  <si>
+    <t>87750891040</t>
+  </si>
+  <si>
+    <t>990430401077</t>
+  </si>
+  <si>
+    <t>87776034491</t>
+  </si>
+  <si>
+    <t>910406401616</t>
+  </si>
+  <si>
+    <t>87027227057</t>
+  </si>
+  <si>
+    <t>940621402511</t>
+  </si>
+  <si>
+    <t>87052148869</t>
+  </si>
+  <si>
+    <t>870727402898</t>
+  </si>
+  <si>
+    <t>87021929309</t>
+  </si>
+  <si>
+    <t>970322400444</t>
+  </si>
+  <si>
+    <t>87071415060</t>
+  </si>
+  <si>
+    <t>870111401933</t>
+  </si>
+  <si>
+    <t>87754000689</t>
+  </si>
+  <si>
+    <t>890202402748</t>
+  </si>
+  <si>
+    <t>87057152409</t>
+  </si>
+  <si>
+    <t>770121401795</t>
+  </si>
+  <si>
+    <t>87713651991</t>
+  </si>
+  <si>
+    <t>910720401504</t>
+  </si>
+  <si>
+    <t>87716746351</t>
+  </si>
+  <si>
+    <t>870131401582</t>
+  </si>
+  <si>
+    <t>87713221595</t>
+  </si>
+  <si>
+    <t>880114401274</t>
+  </si>
+  <si>
+    <t>87073202420</t>
+  </si>
+  <si>
+    <t>990816401570</t>
+  </si>
+  <si>
+    <t>87025097257</t>
+  </si>
+  <si>
+    <t>870901402239</t>
+  </si>
+  <si>
+    <t>87710506398</t>
+  </si>
+  <si>
+    <t>960204451564</t>
+  </si>
+  <si>
+    <t>87712624855</t>
+  </si>
+  <si>
+    <t>810923402075</t>
   </si>
 </sst>
 </file>
@@ -3711,7 +4038,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03590B70-E5C8-4C4E-BF58-0C7B00876EA6}">
-  <dimension ref="A1:H326"/>
+  <dimension ref="A1:H366"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42.33203125" bestFit="1" customWidth="1"/>
@@ -12199,6 +12526,1046 @@
         <v>52</v>
       </c>
     </row>
+    <row r="327" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A327" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B327">
+        <v>11</v>
+      </c>
+      <c r="C327" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D327" t="s">
+        <v>1168</v>
+      </c>
+      <c r="E327" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F327">
+        <v>132276</v>
+      </c>
+      <c r="G327" t="s">
+        <v>972</v>
+      </c>
+      <c r="H327" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="328" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A328" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B328">
+        <v>15</v>
+      </c>
+      <c r="C328" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D328" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E328" t="s">
+        <v>1171</v>
+      </c>
+      <c r="F328">
+        <v>132276</v>
+      </c>
+      <c r="G328" t="s">
+        <v>972</v>
+      </c>
+      <c r="H328" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="329" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A329" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B329">
+        <v>13</v>
+      </c>
+      <c r="C329" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D329" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E329" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F329">
+        <v>132276</v>
+      </c>
+      <c r="G329" t="s">
+        <v>972</v>
+      </c>
+      <c r="H329" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="330" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A330" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B330">
+        <v>11</v>
+      </c>
+      <c r="C330" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D330" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E330" t="s">
+        <v>1175</v>
+      </c>
+      <c r="F330">
+        <v>132276</v>
+      </c>
+      <c r="G330" t="s">
+        <v>972</v>
+      </c>
+      <c r="H330" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="331" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A331" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B331">
+        <v>10</v>
+      </c>
+      <c r="C331" t="s">
+        <v>1149</v>
+      </c>
+      <c r="D331" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E331" t="s">
+        <v>1177</v>
+      </c>
+      <c r="F331">
+        <v>132276</v>
+      </c>
+      <c r="G331" t="s">
+        <v>972</v>
+      </c>
+      <c r="H331" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="332" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A332" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B332">
+        <v>9</v>
+      </c>
+      <c r="C332" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D332" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E332" t="s">
+        <v>1175</v>
+      </c>
+      <c r="F332">
+        <v>132276</v>
+      </c>
+      <c r="G332" t="s">
+        <v>972</v>
+      </c>
+      <c r="H332" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="333" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A333" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B333">
+        <v>8</v>
+      </c>
+      <c r="C333" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D333" t="s">
+        <v>1168</v>
+      </c>
+      <c r="E333" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F333">
+        <v>132276</v>
+      </c>
+      <c r="G333" t="s">
+        <v>972</v>
+      </c>
+      <c r="H333" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="334" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A334" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B334">
+        <v>5</v>
+      </c>
+      <c r="C334" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D334" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E334" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F334">
+        <v>132276</v>
+      </c>
+      <c r="G334" t="s">
+        <v>972</v>
+      </c>
+      <c r="H334" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="335" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A335" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B335">
+        <v>5</v>
+      </c>
+      <c r="C335" t="s">
+        <v>1151</v>
+      </c>
+      <c r="D335" t="s">
+        <v>1180</v>
+      </c>
+      <c r="E335" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F335">
+        <v>132276</v>
+      </c>
+      <c r="G335" t="s">
+        <v>972</v>
+      </c>
+      <c r="H335" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="336" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A336" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B336">
+        <v>6</v>
+      </c>
+      <c r="C336" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D336" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E336" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F336">
+        <v>132276</v>
+      </c>
+      <c r="G336" t="s">
+        <v>972</v>
+      </c>
+      <c r="H336" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="337" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A337" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B337">
+        <v>6</v>
+      </c>
+      <c r="C337" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D337" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E337" t="s">
+        <v>1171</v>
+      </c>
+      <c r="F337">
+        <v>132276</v>
+      </c>
+      <c r="G337" t="s">
+        <v>972</v>
+      </c>
+      <c r="H337" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="338" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A338" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B338">
+        <v>6</v>
+      </c>
+      <c r="C338" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D338" t="s">
+        <v>1182</v>
+      </c>
+      <c r="E338" t="s">
+        <v>1183</v>
+      </c>
+      <c r="F338">
+        <v>132276</v>
+      </c>
+      <c r="G338" t="s">
+        <v>972</v>
+      </c>
+      <c r="H338" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="339" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A339" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B339">
+        <v>8</v>
+      </c>
+      <c r="C339" t="s">
+        <v>1153</v>
+      </c>
+      <c r="D339" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E339" t="s">
+        <v>1185</v>
+      </c>
+      <c r="F339">
+        <v>132276</v>
+      </c>
+      <c r="G339" t="s">
+        <v>972</v>
+      </c>
+      <c r="H339" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="340" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A340" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B340">
+        <v>7</v>
+      </c>
+      <c r="C340" t="s">
+        <v>1153</v>
+      </c>
+      <c r="D340" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E340" t="s">
+        <v>1185</v>
+      </c>
+      <c r="F340">
+        <v>132276</v>
+      </c>
+      <c r="G340" t="s">
+        <v>972</v>
+      </c>
+      <c r="H340" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="341" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A341" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B341">
+        <v>7</v>
+      </c>
+      <c r="C341" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D341" t="s">
+        <v>1168</v>
+      </c>
+      <c r="E341" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F341">
+        <v>132276</v>
+      </c>
+      <c r="G341" t="s">
+        <v>972</v>
+      </c>
+      <c r="H341" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="342" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A342" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B342">
+        <v>10</v>
+      </c>
+      <c r="C342" t="s">
+        <v>1154</v>
+      </c>
+      <c r="D342" t="s">
+        <v>1186</v>
+      </c>
+      <c r="E342" t="s">
+        <v>1187</v>
+      </c>
+      <c r="F342">
+        <v>132277</v>
+      </c>
+      <c r="G342" t="s">
+        <v>899</v>
+      </c>
+      <c r="H342" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="343" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A343" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B343">
+        <v>10</v>
+      </c>
+      <c r="C343" t="s">
+        <v>1155</v>
+      </c>
+      <c r="D343" t="s">
+        <v>1188</v>
+      </c>
+      <c r="E343" t="s">
+        <v>1189</v>
+      </c>
+      <c r="F343">
+        <v>132277</v>
+      </c>
+      <c r="G343" t="s">
+        <v>899</v>
+      </c>
+      <c r="H343" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="344" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A344" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B344">
+        <v>14</v>
+      </c>
+      <c r="C344" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D344" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E344" t="s">
+        <v>1191</v>
+      </c>
+      <c r="F344">
+        <v>132277</v>
+      </c>
+      <c r="G344" t="s">
+        <v>899</v>
+      </c>
+      <c r="H344" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="345" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A345" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B345">
+        <v>11</v>
+      </c>
+      <c r="C345" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D345" t="s">
+        <v>1192</v>
+      </c>
+      <c r="E345" t="s">
+        <v>1193</v>
+      </c>
+      <c r="F345">
+        <v>132277</v>
+      </c>
+      <c r="G345" t="s">
+        <v>899</v>
+      </c>
+      <c r="H345" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="346" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A346" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B346">
+        <v>10</v>
+      </c>
+      <c r="C346" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D346" t="s">
+        <v>1192</v>
+      </c>
+      <c r="E346" t="s">
+        <v>1193</v>
+      </c>
+      <c r="F346">
+        <v>132277</v>
+      </c>
+      <c r="G346" t="s">
+        <v>899</v>
+      </c>
+      <c r="H346" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="347" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A347" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B347">
+        <v>14</v>
+      </c>
+      <c r="C347" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D347" t="s">
+        <v>1194</v>
+      </c>
+      <c r="E347" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F347">
+        <v>132277</v>
+      </c>
+      <c r="G347" t="s">
+        <v>899</v>
+      </c>
+      <c r="H347" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="348" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A348" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B348">
+        <v>16</v>
+      </c>
+      <c r="C348" t="s">
+        <v>1159</v>
+      </c>
+      <c r="D348" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E348" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F348">
+        <v>132277</v>
+      </c>
+      <c r="G348" t="s">
+        <v>899</v>
+      </c>
+      <c r="H348" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="349" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A349" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B349">
+        <v>16</v>
+      </c>
+      <c r="C349" t="s">
+        <v>1160</v>
+      </c>
+      <c r="D349" t="s">
+        <v>1198</v>
+      </c>
+      <c r="E349" t="s">
+        <v>1199</v>
+      </c>
+      <c r="F349">
+        <v>132277</v>
+      </c>
+      <c r="G349" t="s">
+        <v>899</v>
+      </c>
+      <c r="H349" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="350" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A350" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B350">
+        <v>12</v>
+      </c>
+      <c r="C350" t="s">
+        <v>1161</v>
+      </c>
+      <c r="D350" t="s">
+        <v>1200</v>
+      </c>
+      <c r="E350" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F350">
+        <v>132277</v>
+      </c>
+      <c r="G350" t="s">
+        <v>899</v>
+      </c>
+      <c r="H350" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="351" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A351" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B351">
+        <v>12</v>
+      </c>
+      <c r="C351" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D351" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E351" t="s">
+        <v>1191</v>
+      </c>
+      <c r="F351">
+        <v>132277</v>
+      </c>
+      <c r="G351" t="s">
+        <v>899</v>
+      </c>
+      <c r="H351" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="352" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A352" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B352">
+        <v>15</v>
+      </c>
+      <c r="C352" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D352" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E352" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F352">
+        <v>132277</v>
+      </c>
+      <c r="G352" t="s">
+        <v>899</v>
+      </c>
+      <c r="H352" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="353" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A353" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B353">
+        <v>12</v>
+      </c>
+      <c r="C353" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D353" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E353" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F353">
+        <v>132277</v>
+      </c>
+      <c r="G353" t="s">
+        <v>899</v>
+      </c>
+      <c r="H353" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="354" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A354" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B354">
+        <v>6</v>
+      </c>
+      <c r="C354" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D354" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E354" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F354">
+        <v>133885</v>
+      </c>
+      <c r="G354" t="s">
+        <v>288</v>
+      </c>
+      <c r="H354" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="355" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A355" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B355">
+        <v>5</v>
+      </c>
+      <c r="C355" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D355" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E355" t="s">
+        <v>1207</v>
+      </c>
+      <c r="F355">
+        <v>133885</v>
+      </c>
+      <c r="G355" t="s">
+        <v>288</v>
+      </c>
+      <c r="H355" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="356" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A356" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B356">
+        <v>7</v>
+      </c>
+      <c r="C356" t="s">
+        <v>1165</v>
+      </c>
+      <c r="D356" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E356" t="s">
+        <v>1209</v>
+      </c>
+      <c r="F356">
+        <v>133885</v>
+      </c>
+      <c r="G356" t="s">
+        <v>288</v>
+      </c>
+      <c r="H356" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="357" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A357" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B357">
+        <v>10</v>
+      </c>
+      <c r="C357" t="s">
+        <v>1149</v>
+      </c>
+      <c r="D357" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E357" t="s">
+        <v>1177</v>
+      </c>
+      <c r="F357">
+        <v>133885</v>
+      </c>
+      <c r="G357" t="s">
+        <v>288</v>
+      </c>
+      <c r="H357" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="358" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A358" t="s">
+        <v>1136</v>
+      </c>
+      <c r="B358">
+        <v>8</v>
+      </c>
+      <c r="C358" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D358" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E358" t="s">
+        <v>1191</v>
+      </c>
+      <c r="F358">
+        <v>133885</v>
+      </c>
+      <c r="G358" t="s">
+        <v>288</v>
+      </c>
+      <c r="H358" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="359" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A359" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B359">
+        <v>8</v>
+      </c>
+      <c r="C359" t="s">
+        <v>1166</v>
+      </c>
+      <c r="D359" t="s">
+        <v>1210</v>
+      </c>
+      <c r="E359" t="s">
+        <v>1211</v>
+      </c>
+      <c r="F359">
+        <v>133885</v>
+      </c>
+      <c r="G359" t="s">
+        <v>288</v>
+      </c>
+      <c r="H359" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="360" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A360" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B360">
+        <v>8</v>
+      </c>
+      <c r="C360" t="s">
+        <v>1151</v>
+      </c>
+      <c r="D360" t="s">
+        <v>1180</v>
+      </c>
+      <c r="E360" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F360">
+        <v>133885</v>
+      </c>
+      <c r="G360" t="s">
+        <v>288</v>
+      </c>
+      <c r="H360" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="361" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A361" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B361">
+        <v>8</v>
+      </c>
+      <c r="C361" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D361" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E361" t="s">
+        <v>1207</v>
+      </c>
+      <c r="F361">
+        <v>133885</v>
+      </c>
+      <c r="G361" t="s">
+        <v>288</v>
+      </c>
+      <c r="H361" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="362" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A362" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B362">
+        <v>15</v>
+      </c>
+      <c r="C362" t="s">
+        <v>1165</v>
+      </c>
+      <c r="D362" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E362" t="s">
+        <v>1209</v>
+      </c>
+      <c r="F362">
+        <v>133885</v>
+      </c>
+      <c r="G362" t="s">
+        <v>288</v>
+      </c>
+      <c r="H362" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="363" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A363" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B363">
+        <v>11</v>
+      </c>
+      <c r="C363" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D363" t="s">
+        <v>1212</v>
+      </c>
+      <c r="E363" t="s">
+        <v>1213</v>
+      </c>
+      <c r="F363">
+        <v>133885</v>
+      </c>
+      <c r="G363" t="s">
+        <v>288</v>
+      </c>
+      <c r="H363" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="364" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A364" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B364">
+        <v>11</v>
+      </c>
+      <c r="C364" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D364" t="s">
+        <v>1212</v>
+      </c>
+      <c r="E364" t="s">
+        <v>1213</v>
+      </c>
+      <c r="F364">
+        <v>133885</v>
+      </c>
+      <c r="G364" t="s">
+        <v>288</v>
+      </c>
+      <c r="H364" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="365" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A365" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B365">
+        <v>12</v>
+      </c>
+      <c r="C365" t="s">
+        <v>1159</v>
+      </c>
+      <c r="D365" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E365" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F365">
+        <v>133885</v>
+      </c>
+      <c r="G365" t="s">
+        <v>288</v>
+      </c>
+      <c r="H365" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="366" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A366" t="s">
+        <v>1144</v>
+      </c>
+      <c r="B366">
+        <v>12</v>
+      </c>
+      <c r="C366" t="s">
+        <v>1154</v>
+      </c>
+      <c r="D366" t="s">
+        <v>1186</v>
+      </c>
+      <c r="E366" t="s">
+        <v>1187</v>
+      </c>
+      <c r="F366">
+        <v>133885</v>
+      </c>
+      <c r="G366" t="s">
+        <v>288</v>
+      </c>
+      <c r="H366" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>